<commit_message>
Improve beginner workflows and source-based engineering demand in V5.5.6
Synchronize both platforms, offline tutorial and equipment templates. Preserve historical engineering reports, releases, author credit and licensing. Native release workflows publish only after platform acceptance passes.
</commit_message>
<xml_diff>
--- a/macos/facility_studio/resources/Equipment_Template.xlsx
+++ b/macos/facility_studio/resources/Equipment_Template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填寫說明" sheetId="1" r:id="Rff8c74e5c55c4493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="電力" sheetId="2" r:id="R336edde2b4184f72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCW" sheetId="3" r:id="Re75d9c6d20ed4ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CDA" sheetId="4" r:id="Rd689d976eb384490"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="N2" sheetId="5" r:id="R49cbac2293ea443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXHAUST" sheetId="6" r:id="Rfb63e0629a7b4f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DI" sheetId="7" r:id="Rce03d628ccd84ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PV" sheetId="8" r:id="R904c204c88b04736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填寫說明" sheetId="1" r:id="R441bc35e032444c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="電力" sheetId="2" r:id="R1a4424d21c334066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCW" sheetId="3" r:id="R5515ae00b3f34972"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CDA" sheetId="4" r:id="R75745cf33ca641fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="N2" sheetId="5" r:id="R83f3b60c751b42b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXHAUST" sheetId="6" r:id="R5953b5a207734cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DI" sheetId="7" r:id="R6290b9aff7734a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PV" sheetId="8" r:id="R0a4147711d164c50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -138,7 +138,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -148,7 +148,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -158,7 +158,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -168,7 +168,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -178,7 +178,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -188,7 +188,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -198,7 +198,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -208,7 +208,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -218,7 +218,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -228,7 +228,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -238,7 +238,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -248,7 +248,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -258,7 +258,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -268,7 +268,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -278,7 +278,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -288,7 +288,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -298,7 +298,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -308,7 +308,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -318,7 +318,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -328,7 +328,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -338,7 +338,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -348,7 +348,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -358,7 +358,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -368,7 +368,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -378,7 +378,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -388,7 +388,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -398,7 +398,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -408,7 +408,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -418,7 +418,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -428,7 +428,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -438,7 +438,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -448,7 +448,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -458,7 +458,7 @@
         <x:color rgb="FFAF2D2D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE4DF"/>
         </x:patternFill>
       </x:fill>
@@ -717,7 +717,7 @@
         <x:v>同時使用率</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>填0~100的瞬間同時需求係數。空白採100%。不能用每小時運轉比例替代安全系統的設計量。</x:v>
+        <x:v>50 或 50% 都表示 50%；一般格式數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算，明細會列採用值。空白採 100%。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -3286,7 +3286,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -5451,7 +5451,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8125,7 +8125,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -10815,7 +10815,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -13065,7 +13065,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -15208,7 +15208,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -17780,7 +17780,7 @@
         <x:v>同時使用率(%)</x:v>
       </x:c>
       <x:c r="B113" s="1" t="str">
-        <x:v>瞬間同時需求的估算係數，填0~100；不是每小時運轉分鐘數。支路仍按額定負載。</x:v>
+        <x:v>50 或 50% 表示 50%；一般數值 0.5 表示 0.5%。Excel 百分比格式依顯示比例換算；不是每小時運轉比例。支路仍核全載。</x:v>
       </x:c>
     </x:row>
     <x:row r="114">

</xml_diff>